<commit_message>
TImetable generate same every time fixes
</commit_message>
<xml_diff>
--- a/educhrono-backend/app/templates/Teacherload_final.xlsx
+++ b/educhrono-backend/app/templates/Teacherload_final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\FunctionX\educhrono\educhrono-backend\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DCCA0D1-41D3-485D-ADAE-2580A0C30609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55E48471-229E-4C7F-85E6-B702A9BA297A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="100" yWindow="0" windowWidth="19100" windowHeight="10800" xr2:uid="{0DA5C644-9AF4-4DA6-AF46-A5CC77FF4A05}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="185">
   <si>
     <t>L</t>
   </si>
@@ -1037,7 +1037,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2242A443-A87D-4EF6-BCEE-CBEFCE842B53}">
-  <dimension ref="A1:L133"/>
+  <dimension ref="A1:L121"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.54296875" customWidth="1"/>
@@ -5446,7 +5446,7 @@
         <v>3</v>
       </c>
       <c r="H116" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I116" s="2" t="s">
         <v>8</v>
@@ -5484,7 +5484,7 @@
         <v>3</v>
       </c>
       <c r="H117" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I117" s="2" t="s">
         <v>8</v>
@@ -5522,7 +5522,7 @@
         <v>3</v>
       </c>
       <c r="H118" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I118" s="2" t="s">
         <v>8</v>
@@ -5560,7 +5560,7 @@
         <v>3</v>
       </c>
       <c r="H119" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I119" s="2" t="s">
         <v>8</v>
@@ -5598,7 +5598,7 @@
         <v>3</v>
       </c>
       <c r="H120" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I120" s="2" t="s">
         <v>8</v>
@@ -5636,7 +5636,7 @@
         <v>3</v>
       </c>
       <c r="H121" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I121" s="2" t="s">
         <v>8</v>
@@ -5648,462 +5648,6 @@
         <v>184</v>
       </c>
       <c r="L121" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A122" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B122" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C122" s="2">
-        <v>0</v>
-      </c>
-      <c r="D122" s="2">
-        <v>0</v>
-      </c>
-      <c r="E122" s="2">
-        <v>0</v>
-      </c>
-      <c r="F122" s="2">
-        <v>2</v>
-      </c>
-      <c r="G122" s="2">
-        <v>0</v>
-      </c>
-      <c r="H122" s="2">
-        <v>7</v>
-      </c>
-      <c r="I122" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J122" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="K122" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="L122" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A123" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B123" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C123" s="2">
-        <v>0</v>
-      </c>
-      <c r="D123" s="2">
-        <v>0</v>
-      </c>
-      <c r="E123" s="2">
-        <v>0</v>
-      </c>
-      <c r="F123" s="2">
-        <v>2</v>
-      </c>
-      <c r="G123" s="2">
-        <v>0</v>
-      </c>
-      <c r="H123" s="2">
-        <v>7</v>
-      </c>
-      <c r="I123" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J123" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="K123" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="L123" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A124" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B124" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C124" s="2">
-        <v>0</v>
-      </c>
-      <c r="D124" s="2">
-        <v>0</v>
-      </c>
-      <c r="E124" s="2">
-        <v>0</v>
-      </c>
-      <c r="F124" s="2">
-        <v>2</v>
-      </c>
-      <c r="G124" s="2">
-        <v>0</v>
-      </c>
-      <c r="H124" s="2">
-        <v>7</v>
-      </c>
-      <c r="I124" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J124" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="K124" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="L124" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A125" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B125" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C125" s="2">
-        <v>0</v>
-      </c>
-      <c r="D125" s="2">
-        <v>0</v>
-      </c>
-      <c r="E125" s="2">
-        <v>0</v>
-      </c>
-      <c r="F125" s="2">
-        <v>2</v>
-      </c>
-      <c r="G125" s="2">
-        <v>0</v>
-      </c>
-      <c r="H125" s="2">
-        <v>7</v>
-      </c>
-      <c r="I125" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J125" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="K125" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="L125" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A126" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B126" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C126" s="2">
-        <v>0</v>
-      </c>
-      <c r="D126" s="2">
-        <v>0</v>
-      </c>
-      <c r="E126" s="2">
-        <v>0</v>
-      </c>
-      <c r="F126" s="2">
-        <v>2</v>
-      </c>
-      <c r="G126" s="2">
-        <v>0</v>
-      </c>
-      <c r="H126" s="2">
-        <v>7</v>
-      </c>
-      <c r="I126" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J126" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="K126" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="L126" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A127" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B127" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C127" s="2">
-        <v>0</v>
-      </c>
-      <c r="D127" s="2">
-        <v>0</v>
-      </c>
-      <c r="E127" s="2">
-        <v>0</v>
-      </c>
-      <c r="F127" s="2">
-        <v>2</v>
-      </c>
-      <c r="G127" s="2">
-        <v>0</v>
-      </c>
-      <c r="H127" s="2">
-        <v>7</v>
-      </c>
-      <c r="I127" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J127" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="K127" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="L127" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A128" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B128" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="C128" s="2">
-        <v>0</v>
-      </c>
-      <c r="D128" s="2">
-        <v>0</v>
-      </c>
-      <c r="E128" s="2">
-        <v>0</v>
-      </c>
-      <c r="F128" s="2">
-        <v>0</v>
-      </c>
-      <c r="G128" s="2">
-        <v>3</v>
-      </c>
-      <c r="H128" s="2">
-        <v>5</v>
-      </c>
-      <c r="I128" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J128" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="K128" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="L128" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A129" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B129" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="C129" s="2">
-        <v>0</v>
-      </c>
-      <c r="D129" s="2">
-        <v>0</v>
-      </c>
-      <c r="E129" s="2">
-        <v>0</v>
-      </c>
-      <c r="F129" s="2">
-        <v>0</v>
-      </c>
-      <c r="G129" s="2">
-        <v>3</v>
-      </c>
-      <c r="H129" s="2">
-        <v>5</v>
-      </c>
-      <c r="I129" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J129" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="K129" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="L129" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A130" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B130" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="C130" s="2">
-        <v>0</v>
-      </c>
-      <c r="D130" s="2">
-        <v>0</v>
-      </c>
-      <c r="E130" s="2">
-        <v>0</v>
-      </c>
-      <c r="F130" s="2">
-        <v>0</v>
-      </c>
-      <c r="G130" s="2">
-        <v>3</v>
-      </c>
-      <c r="H130" s="2">
-        <v>5</v>
-      </c>
-      <c r="I130" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J130" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="K130" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="L130" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A131" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B131" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="C131" s="2">
-        <v>0</v>
-      </c>
-      <c r="D131" s="2">
-        <v>0</v>
-      </c>
-      <c r="E131" s="2">
-        <v>0</v>
-      </c>
-      <c r="F131" s="2">
-        <v>0</v>
-      </c>
-      <c r="G131" s="2">
-        <v>3</v>
-      </c>
-      <c r="H131" s="2">
-        <v>5</v>
-      </c>
-      <c r="I131" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J131" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="K131" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="L131" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A132" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B132" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="C132" s="2">
-        <v>0</v>
-      </c>
-      <c r="D132" s="2">
-        <v>0</v>
-      </c>
-      <c r="E132" s="2">
-        <v>0</v>
-      </c>
-      <c r="F132" s="2">
-        <v>0</v>
-      </c>
-      <c r="G132" s="2">
-        <v>3</v>
-      </c>
-      <c r="H132" s="2">
-        <v>5</v>
-      </c>
-      <c r="I132" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J132" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="K132" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="L132" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A133" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B133" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="C133" s="2">
-        <v>0</v>
-      </c>
-      <c r="D133" s="2">
-        <v>0</v>
-      </c>
-      <c r="E133" s="2">
-        <v>0</v>
-      </c>
-      <c r="F133" s="2">
-        <v>0</v>
-      </c>
-      <c r="G133" s="2">
-        <v>3</v>
-      </c>
-      <c r="H133" s="2">
-        <v>5</v>
-      </c>
-      <c r="I133" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J133" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="K133" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="L133" s="2" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>